<commit_message>
feat: Add DRM Rapid Screening Tool questionnaire data.
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Questionnaire.xlsx
+++ b/data/DRM Rapid Screening Tool - Questionnaire.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="80">
   <si>
     <t xml:space="preserve">Evaluating Disaster Risk Management Policy Frameworks: A Rapid Screening Tool</t>
   </si>
@@ -87,9 +87,6 @@
     <t xml:space="preserve">Is there a legal framework (e.g., a DRM law or other legally-binding instruments) defining distinct responsibilities for disaster risk reduction and emergency management?</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes</t>
-  </si>
-  <si>
     <t xml:space="preserve">Have any implementing decrees or regulations been approved since the adoption of the DRM legal framework? (e.g., rules on the structure or functions of the DRM agency or implementing regulations of the DRM law)</t>
   </si>
   <si>
@@ -181,9 +178,6 @@
   </si>
   <si>
     <t xml:space="preserve">Have any watershed basins undergone improvements in water management in the last four years?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partially</t>
   </si>
   <si>
     <t xml:space="preserve">4. Preparedness</t>
@@ -1067,7 +1061,7 @@
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="18" t="str">
         <f aca="false">IF(COUNTBLANK(E15:E60)&gt;0,_xlfn.CONCAT("Please complete the assessment to proceed. Remaining questions: ",COUNTBLANK(E15:E60)), _xlfn.TEXTJOIN("&amp;",FALSE(),K15:K60))</f>
-        <v>Q1;Yes;1&amp;Q2;Yes;1&amp;Q3;Yes;1&amp;Q4;Yes;1&amp;Q5;Yes;1&amp;Q6;Yes;1&amp;Q7;Yes;1&amp;Q8;Yes;1&amp;Q9;Yes;1&amp;Q10;Yes;1&amp;Q11;Yes;1&amp;Q12;Yes;1&amp;Q13;Yes;1&amp;Q14;Yes;1&amp;Q15;Yes;1&amp;Q16;Yes;1&amp;Q17;Yes;1&amp;Q18;Yes;0.25&amp;Q19;Yes;0.25&amp;Q20;Yes;0.25&amp;Q21;Yes;0.25&amp;Q22;Yes;1&amp;Q23;Yes;1&amp;Q24;Yes;1&amp;Q25;Yes;1&amp;Q26;Partially;1&amp;Q27;Partially;1&amp;Q28;Yes;1&amp;Q29;Yes;1&amp;Q30;Yes;1&amp;Q31;Yes;1&amp;Q32;Yes;1&amp;Q33;Yes;1&amp;Q34;Yes;1&amp;Q35;Yes;1&amp;Q36;Yes;1&amp;Q37;Yes;1&amp;Q38;Yes;1&amp;Q39;Yes;1&amp;Q40;Yes;1&amp;Q41;Yes;1&amp;Q42;Yes;1&amp;Q43;Yes;1&amp;Q44;Yes;1&amp;Q45;Yes;1&amp;Q46;Yes;1</v>
+        <v>Please complete the assessment to proceed. Remaining questions: 46</v>
       </c>
       <c r="C10" s="19"/>
       <c r="D10" s="20"/>
@@ -1175,9 +1169,7 @@
       <c r="D15" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="E15" s="26" t="s">
-        <v>21</v>
-      </c>
+      <c r="E15" s="26"/>
       <c r="F15" s="26"/>
       <c r="G15" s="26"/>
       <c r="H15" s="26" t="n">
@@ -1192,18 +1184,16 @@
       </c>
       <c r="K15" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J15,E15,H15)</f>
-        <v>Q1;Yes;1</v>
+        <v>Q1;;1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="24"/>
       <c r="C16" s="24"/>
       <c r="D16" s="28" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" s="29" t="s">
         <v>21</v>
       </c>
+      <c r="E16" s="29"/>
       <c r="F16" s="29"/>
       <c r="G16" s="29"/>
       <c r="H16" s="30" t="n">
@@ -1219,7 +1209,7 @@
       </c>
       <c r="K16" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J16,E16,H16)</f>
-        <v>Q2;Yes;1</v>
+        <v>Q2;;1</v>
       </c>
       <c r="L16" s="32"/>
     </row>
@@ -1227,11 +1217,9 @@
       <c r="B17" s="24"/>
       <c r="C17" s="24"/>
       <c r="D17" s="25" t="s">
-        <v>23</v>
-      </c>
-      <c r="E17" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="E17" s="26"/>
       <c r="F17" s="26"/>
       <c r="G17" s="26"/>
       <c r="H17" s="26" t="n">
@@ -1247,18 +1235,16 @@
       </c>
       <c r="K17" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J17,E17,H17)</f>
-        <v>Q3;Yes;1</v>
+        <v>Q3;;1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B18" s="24"/>
       <c r="C18" s="24"/>
       <c r="D18" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="E18" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="E18" s="29"/>
       <c r="F18" s="29"/>
       <c r="G18" s="29"/>
       <c r="H18" s="30" t="n">
@@ -1274,20 +1260,18 @@
       </c>
       <c r="K18" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J18,E18,H18)</f>
-        <v>Q4;Yes;1</v>
+        <v>Q4;;1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="24"/>
       <c r="C19" s="24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D19" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="E19" s="26" t="s">
-        <v>21</v>
-      </c>
+      <c r="E19" s="26"/>
       <c r="F19" s="26"/>
       <c r="G19" s="26"/>
       <c r="H19" s="26" t="n">
@@ -1303,18 +1287,16 @@
       </c>
       <c r="K19" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J19,E19,H19)</f>
-        <v>Q5;Yes;1</v>
+        <v>Q5;;1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="24"/>
       <c r="C20" s="24"/>
       <c r="D20" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="E20" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="E20" s="29"/>
       <c r="F20" s="29"/>
       <c r="G20" s="29"/>
       <c r="H20" s="30" t="n">
@@ -1330,23 +1312,21 @@
       </c>
       <c r="K20" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J20,E20,H20)</f>
-        <v>Q6;Yes;1</v>
+        <v>Q6;;1</v>
       </c>
       <c r="L20" s="33"/>
     </row>
     <row r="21" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B21" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C21" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="C21" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="E21" s="26" t="s">
-        <v>21</v>
-      </c>
+      <c r="E21" s="26"/>
       <c r="F21" s="26"/>
       <c r="G21" s="26"/>
       <c r="H21" s="26" t="n">
@@ -1362,18 +1342,16 @@
       </c>
       <c r="K21" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J21,E21,H21)</f>
-        <v>Q7;Yes;1</v>
+        <v>Q7;;1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="24"/>
       <c r="C22" s="24"/>
       <c r="D22" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="E22" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="E22" s="29"/>
       <c r="F22" s="29"/>
       <c r="G22" s="29"/>
       <c r="H22" s="30" t="n">
@@ -1389,18 +1367,16 @@
       </c>
       <c r="K22" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J22,E22,H22)</f>
-        <v>Q8;Yes;1</v>
+        <v>Q8;;1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="24"/>
       <c r="C23" s="24"/>
       <c r="D23" s="25" t="s">
-        <v>31</v>
-      </c>
-      <c r="E23" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E23" s="26"/>
       <c r="F23" s="26"/>
       <c r="G23" s="26"/>
       <c r="H23" s="26" t="n">
@@ -1416,7 +1392,7 @@
       </c>
       <c r="K23" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J23,E23,H23)</f>
-        <v>Q9;Yes;1</v>
+        <v>Q9;;1</v>
       </c>
       <c r="L23" s="32"/>
     </row>
@@ -1424,11 +1400,9 @@
       <c r="B24" s="24"/>
       <c r="C24" s="24"/>
       <c r="D24" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="E24" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="E24" s="29"/>
       <c r="F24" s="29"/>
       <c r="G24" s="29"/>
       <c r="H24" s="30" t="n">
@@ -1444,22 +1418,20 @@
       </c>
       <c r="K24" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J24,E24,H24)</f>
-        <v>Q10;Yes;1</v>
+        <v>Q10;;1</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25" s="24" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="D25" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="D25" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="E25" s="26" t="s">
-        <v>21</v>
-      </c>
+      <c r="E25" s="26"/>
       <c r="F25" s="26"/>
       <c r="G25" s="26"/>
       <c r="H25" s="26" t="n">
@@ -1475,18 +1447,16 @@
       </c>
       <c r="K25" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J25,E25,H25)</f>
-        <v>Q11;Yes;1</v>
+        <v>Q11;;1</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="24"/>
       <c r="C26" s="24"/>
       <c r="D26" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="E26" s="29"/>
       <c r="F26" s="29"/>
       <c r="G26" s="29"/>
       <c r="H26" s="30" t="n">
@@ -1502,18 +1472,16 @@
       </c>
       <c r="K26" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J26,E26,H26)</f>
-        <v>Q12;Yes;1</v>
+        <v>Q12;;1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="24"/>
       <c r="C27" s="24"/>
       <c r="D27" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="E27" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="E27" s="26"/>
       <c r="F27" s="26"/>
       <c r="G27" s="26"/>
       <c r="H27" s="26" t="n">
@@ -1529,18 +1497,16 @@
       </c>
       <c r="K27" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J27,E27,H27)</f>
-        <v>Q13;Yes;1</v>
+        <v>Q13;;1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="24"/>
       <c r="C28" s="24"/>
       <c r="D28" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="E28" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="E28" s="29"/>
       <c r="F28" s="29"/>
       <c r="G28" s="29"/>
       <c r="H28" s="30" t="n">
@@ -1556,21 +1522,19 @@
       </c>
       <c r="K28" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J28,E28,H28)</f>
-        <v>Q14;Yes;1</v>
+        <v>Q14;;1</v>
       </c>
       <c r="L28" s="32"/>
     </row>
     <row r="29" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="24"/>
       <c r="C29" s="24" t="s">
+        <v>38</v>
+      </c>
+      <c r="D29" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D29" s="25" t="s">
-        <v>40</v>
-      </c>
-      <c r="E29" s="26" t="s">
-        <v>21</v>
-      </c>
+      <c r="E29" s="26"/>
       <c r="F29" s="26"/>
       <c r="G29" s="26"/>
       <c r="H29" s="26" t="n">
@@ -1586,18 +1550,16 @@
       </c>
       <c r="K29" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J29,E29,H29)</f>
-        <v>Q15;Yes;1</v>
+        <v>Q15;;1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="24"/>
       <c r="C30" s="24"/>
       <c r="D30" s="24" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="E30" s="29"/>
       <c r="F30" s="29"/>
       <c r="G30" s="29"/>
       <c r="H30" s="30" t="n">
@@ -1613,18 +1575,16 @@
       </c>
       <c r="K30" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J30,E30,H30)</f>
-        <v>Q16;Yes;1</v>
+        <v>Q16;;1</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B31" s="24"/>
       <c r="C31" s="24"/>
       <c r="D31" s="25" t="s">
-        <v>42</v>
-      </c>
-      <c r="E31" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>41</v>
+      </c>
+      <c r="E31" s="26"/>
       <c r="F31" s="26"/>
       <c r="G31" s="26"/>
       <c r="H31" s="26" t="n">
@@ -1640,21 +1600,19 @@
       </c>
       <c r="K31" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J31,E31,H31)</f>
-        <v>Q17;Yes;1</v>
+        <v>Q17;;1</v>
       </c>
       <c r="L31" s="34"/>
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="24"/>
       <c r="C32" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="D32" s="24" t="s">
         <v>43</v>
       </c>
-      <c r="D32" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="E32" s="29" t="s">
-        <v>21</v>
-      </c>
+      <c r="E32" s="29"/>
       <c r="F32" s="29"/>
       <c r="G32" s="29"/>
       <c r="H32" s="30" t="n">
@@ -1670,18 +1628,16 @@
       </c>
       <c r="K32" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J32,E32,H32)</f>
-        <v>Q18;Yes;0.25</v>
+        <v>Q18;;0.25</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
       <c r="D33" s="35" t="s">
-        <v>45</v>
-      </c>
-      <c r="E33" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="E33" s="26"/>
       <c r="F33" s="26"/>
       <c r="G33" s="26"/>
       <c r="H33" s="26" t="n">
@@ -1697,18 +1653,16 @@
       </c>
       <c r="K33" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J33,E33,H33)</f>
-        <v>Q19;Yes;0.25</v>
+        <v>Q19;;0.25</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="24"/>
       <c r="C34" s="24"/>
       <c r="D34" s="36" t="s">
-        <v>46</v>
-      </c>
-      <c r="E34" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="E34" s="29"/>
       <c r="F34" s="29"/>
       <c r="G34" s="29"/>
       <c r="H34" s="30" t="n">
@@ -1724,18 +1678,16 @@
       </c>
       <c r="K34" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J34,E34,H34)</f>
-        <v>Q20;Yes;0.25</v>
+        <v>Q20;;0.25</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="24"/>
       <c r="C35" s="24"/>
       <c r="D35" s="35" t="s">
-        <v>47</v>
-      </c>
-      <c r="E35" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="E35" s="26"/>
       <c r="F35" s="26"/>
       <c r="G35" s="26"/>
       <c r="H35" s="26" t="n">
@@ -1751,18 +1703,16 @@
       </c>
       <c r="K35" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J35,E35,H35)</f>
-        <v>Q21;Yes;0.25</v>
+        <v>Q21;;0.25</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B36" s="24"/>
       <c r="C36" s="24"/>
       <c r="D36" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="E36" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="E36" s="29"/>
       <c r="F36" s="29"/>
       <c r="G36" s="29"/>
       <c r="H36" s="30" t="n">
@@ -1778,18 +1728,16 @@
       </c>
       <c r="K36" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J36,E36,H36)</f>
-        <v>Q22;Yes;1</v>
+        <v>Q22;;1</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B37" s="24"/>
       <c r="C37" s="24"/>
       <c r="D37" s="25" t="s">
-        <v>49</v>
-      </c>
-      <c r="E37" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="E37" s="26"/>
       <c r="F37" s="26"/>
       <c r="G37" s="26"/>
       <c r="H37" s="26" t="n">
@@ -1805,18 +1753,16 @@
       </c>
       <c r="K37" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J37,E37,H37)</f>
-        <v>Q23;Yes;1</v>
+        <v>Q23;;1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="24"/>
       <c r="C38" s="24"/>
       <c r="D38" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="E38" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="E38" s="29"/>
       <c r="F38" s="29"/>
       <c r="G38" s="29"/>
       <c r="H38" s="30" t="n">
@@ -1832,18 +1778,16 @@
       </c>
       <c r="K38" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J38,E38,H38)</f>
-        <v>Q24;Yes;1</v>
+        <v>Q24;;1</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="24"/>
       <c r="C39" s="24"/>
       <c r="D39" s="25" t="s">
-        <v>51</v>
-      </c>
-      <c r="E39" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="E39" s="26"/>
       <c r="F39" s="26"/>
       <c r="G39" s="26"/>
       <c r="H39" s="26" t="n">
@@ -1859,18 +1803,16 @@
       </c>
       <c r="K39" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J39,E39,H39)</f>
-        <v>Q25;Yes;1</v>
+        <v>Q25;;1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="24"/>
       <c r="C40" s="24"/>
       <c r="D40" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="E40" s="29" t="s">
-        <v>53</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="E40" s="29"/>
       <c r="F40" s="29"/>
       <c r="G40" s="29"/>
       <c r="H40" s="30" t="n">
@@ -1886,22 +1828,20 @@
       </c>
       <c r="K40" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J40,E40,H40)</f>
-        <v>Q26;Partially;1</v>
+        <v>Q26;;1</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="C41" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="D41" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="C41" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="D41" s="38" t="s">
-        <v>56</v>
-      </c>
-      <c r="E41" s="26" t="s">
-        <v>53</v>
-      </c>
+      <c r="E41" s="26"/>
       <c r="F41" s="26"/>
       <c r="G41" s="26"/>
       <c r="H41" s="27" t="n">
@@ -1917,18 +1857,16 @@
       </c>
       <c r="K41" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J41,E41,H41)</f>
-        <v>Q27;Partially;1</v>
+        <v>Q27;;1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="37"/>
       <c r="C42" s="24"/>
       <c r="D42" s="39" t="s">
-        <v>57</v>
-      </c>
-      <c r="E42" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="E42" s="29"/>
       <c r="F42" s="29"/>
       <c r="G42" s="29"/>
       <c r="H42" s="31" t="n">
@@ -1944,18 +1882,16 @@
       </c>
       <c r="K42" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J42,E42,H42)</f>
-        <v>Q28;Yes;1</v>
+        <v>Q28;;1</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B43" s="37"/>
       <c r="C43" s="24"/>
       <c r="D43" s="38" t="s">
-        <v>58</v>
-      </c>
-      <c r="E43" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="E43" s="26"/>
       <c r="F43" s="26"/>
       <c r="G43" s="26"/>
       <c r="H43" s="27" t="n">
@@ -1971,20 +1907,18 @@
       </c>
       <c r="K43" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J43,E43,H43)</f>
-        <v>Q29;Yes;1</v>
+        <v>Q29;;1</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B44" s="37"/>
       <c r="C44" s="24" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D44" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E44" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="E44" s="29"/>
       <c r="F44" s="29"/>
       <c r="G44" s="29"/>
       <c r="H44" s="31" t="n">
@@ -2000,18 +1934,16 @@
       </c>
       <c r="K44" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J44,E44,H44)</f>
-        <v>Q30;Yes;1</v>
+        <v>Q30;;1</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="37"/>
       <c r="C45" s="24"/>
       <c r="D45" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="E45" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="E45" s="26"/>
       <c r="F45" s="26"/>
       <c r="G45" s="26"/>
       <c r="H45" s="27" t="n">
@@ -2027,18 +1959,16 @@
       </c>
       <c r="K45" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J45,E45,H45)</f>
-        <v>Q31;Yes;1</v>
+        <v>Q31;;1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B46" s="37"/>
       <c r="C46" s="24"/>
       <c r="D46" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="E46" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="E46" s="29"/>
       <c r="F46" s="29"/>
       <c r="G46" s="29"/>
       <c r="H46" s="31" t="n">
@@ -2054,18 +1984,16 @@
       </c>
       <c r="K46" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J46,E46,H46)</f>
-        <v>Q32;Yes;1</v>
+        <v>Q32;;1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B47" s="37"/>
       <c r="C47" s="24"/>
       <c r="D47" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="E47" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="E47" s="26"/>
       <c r="F47" s="26"/>
       <c r="G47" s="26"/>
       <c r="H47" s="27" t="n">
@@ -2081,20 +2009,18 @@
       </c>
       <c r="K47" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J47,E47,H47)</f>
-        <v>Q33;Yes;1</v>
+        <v>Q33;;1</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B48" s="37"/>
       <c r="C48" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D48" s="39" t="s">
-        <v>65</v>
-      </c>
-      <c r="E48" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="E48" s="29"/>
       <c r="F48" s="29"/>
       <c r="G48" s="29"/>
       <c r="H48" s="31" t="n">
@@ -2110,18 +2036,16 @@
       </c>
       <c r="K48" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J48,E48,H48)</f>
-        <v>Q34;Yes;1</v>
+        <v>Q34;;1</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B49" s="37"/>
       <c r="C49" s="24"/>
       <c r="D49" s="38" t="s">
-        <v>66</v>
-      </c>
-      <c r="E49" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E49" s="26"/>
       <c r="F49" s="26"/>
       <c r="G49" s="26"/>
       <c r="H49" s="27" t="n">
@@ -2137,18 +2061,16 @@
       </c>
       <c r="K49" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J49,E49,H49)</f>
-        <v>Q35;Yes;1</v>
+        <v>Q35;;1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="37"/>
       <c r="C50" s="24"/>
       <c r="D50" s="39" t="s">
-        <v>67</v>
-      </c>
-      <c r="E50" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="E50" s="29"/>
       <c r="F50" s="29"/>
       <c r="G50" s="29"/>
       <c r="H50" s="31" t="n">
@@ -2164,22 +2086,20 @@
       </c>
       <c r="K50" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J50,E50,H50)</f>
-        <v>Q36;Yes;1</v>
+        <v>Q36;;1</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B51" s="37" t="s">
+        <v>66</v>
+      </c>
+      <c r="C51" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="D51" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="C51" s="24" t="s">
-        <v>69</v>
-      </c>
-      <c r="D51" s="38" t="s">
-        <v>70</v>
-      </c>
-      <c r="E51" s="26" t="s">
-        <v>21</v>
-      </c>
+      <c r="E51" s="26"/>
       <c r="F51" s="26"/>
       <c r="G51" s="26"/>
       <c r="H51" s="27" t="n">
@@ -2195,18 +2115,16 @@
       </c>
       <c r="K51" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J51,E51,H51)</f>
-        <v>Q37;Yes;1</v>
+        <v>Q37;;1</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B52" s="37"/>
       <c r="C52" s="24"/>
       <c r="D52" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="E52" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="E52" s="29"/>
       <c r="F52" s="29"/>
       <c r="G52" s="29"/>
       <c r="H52" s="31" t="n">
@@ -2222,18 +2140,16 @@
       </c>
       <c r="K52" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J52,E52,H52)</f>
-        <v>Q38;Yes;1</v>
+        <v>Q38;;1</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B53" s="37"/>
       <c r="C53" s="24"/>
       <c r="D53" s="38" t="s">
-        <v>72</v>
-      </c>
-      <c r="E53" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="E53" s="26"/>
       <c r="F53" s="26"/>
       <c r="G53" s="26"/>
       <c r="H53" s="27" t="n">
@@ -2249,18 +2165,16 @@
       </c>
       <c r="K53" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J53,E53,H53)</f>
-        <v>Q39;Yes;1</v>
+        <v>Q39;;1</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B54" s="37"/>
       <c r="C54" s="24"/>
       <c r="D54" s="39" t="s">
-        <v>73</v>
-      </c>
-      <c r="E54" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>71</v>
+      </c>
+      <c r="E54" s="29"/>
       <c r="F54" s="29"/>
       <c r="G54" s="29"/>
       <c r="H54" s="31" t="n">
@@ -2276,20 +2190,18 @@
       </c>
       <c r="K54" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J54,E54,H54)</f>
-        <v>Q40;Yes;1</v>
+        <v>Q40;;1</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B55" s="37"/>
       <c r="C55" s="24" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D55" s="38" t="s">
-        <v>75</v>
-      </c>
-      <c r="E55" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="E55" s="26"/>
       <c r="F55" s="26"/>
       <c r="G55" s="26"/>
       <c r="H55" s="27" t="n">
@@ -2305,18 +2217,16 @@
       </c>
       <c r="K55" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J55,E55,H55)</f>
-        <v>Q41;Yes;1</v>
+        <v>Q41;;1</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B56" s="37"/>
       <c r="C56" s="24"/>
       <c r="D56" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="E56" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="E56" s="29"/>
       <c r="F56" s="29"/>
       <c r="G56" s="29"/>
       <c r="H56" s="31" t="n">
@@ -2332,18 +2242,16 @@
       </c>
       <c r="K56" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J56,E56,H56)</f>
-        <v>Q42;Yes;1</v>
+        <v>Q42;;1</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B57" s="37"/>
       <c r="C57" s="24"/>
       <c r="D57" s="38" t="s">
-        <v>77</v>
-      </c>
-      <c r="E57" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="E57" s="26"/>
       <c r="F57" s="26"/>
       <c r="G57" s="26"/>
       <c r="H57" s="27" t="n">
@@ -2359,22 +2267,20 @@
       </c>
       <c r="K57" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J57,E57,H57)</f>
-        <v>Q43;Yes;1</v>
+        <v>Q43;;1</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B58" s="37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C58" s="37" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D58" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="E58" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="E58" s="29"/>
       <c r="F58" s="29"/>
       <c r="G58" s="29"/>
       <c r="H58" s="31" t="n">
@@ -2390,18 +2296,16 @@
       </c>
       <c r="K58" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J58,E58,H58)</f>
-        <v>Q44;Yes;1</v>
+        <v>Q44;;1</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B59" s="37"/>
       <c r="C59" s="37"/>
       <c r="D59" s="38" t="s">
-        <v>80</v>
-      </c>
-      <c r="E59" s="26" t="s">
-        <v>21</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="E59" s="26"/>
       <c r="F59" s="26"/>
       <c r="G59" s="26"/>
       <c r="H59" s="27" t="n">
@@ -2417,18 +2321,16 @@
       </c>
       <c r="K59" s="27" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J59,E59,H59)</f>
-        <v>Q45;Yes;1</v>
+        <v>Q45;;1</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B60" s="37"/>
       <c r="C60" s="37"/>
       <c r="D60" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="E60" s="29" t="s">
-        <v>21</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="E60" s="29"/>
       <c r="F60" s="29"/>
       <c r="G60" s="29"/>
       <c r="H60" s="31" t="n">
@@ -2444,7 +2346,7 @@
       </c>
       <c r="K60" s="30" t="str">
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J60,E60,H60)</f>
-        <v>Q46;Yes;1</v>
+        <v>Q46;;1</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2606,13 +2508,17 @@
     <mergeCell ref="B58:B60"/>
     <mergeCell ref="C58:C60"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E15:G15 E17:G17 E19:G19 E21:G21 E23:G23 E25:G25 E27:G27 E29:G29 E31:G31 E33:G33 E35:G35 E37:G37 E39:G39 E41:G41 E43:G43 E45:G45 E47:G47 E49:G49 E51:G51 E53:G53 E55:G55 E57:G57 E59:G59" type="list">
+  <dataValidations count="3">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E15 E17 E19 E21 E23 E25 E27 E29 E31 E33 E35 E37 E39 E41 E43 E45 E47 E49 E51 E53 E55 E57 E59" type="list">
       <formula1>"Yes,No,Partially,Unknown"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E16:G16 E18:G18 E20:G20 E22:G22 E24:G24 E26:G26 E28:G28 E30:G30 E32:G32 E34:G34 E36:G36 E38:G38 E40:G40 E42:G42 E44:G44 E46:G46 E48:G48 E50:G50 E52:G52 E54:G54 E56:G56 E58:G58 E60:G60" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="E16 E18 E20 E22 E24 E26 E28 E30 E32 E34 E36 E38 E40 E42 E44 E46 E48 E50 E52 E54 E56 E58 E60" type="list">
       <formula1>"Yes,No,Partially,Unknown"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="true" sqref="F15:G60" type="none">
+      <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat: add DRM Rapid Screening Tool questionnaire template
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Questionnaire.xlsx
+++ b/data/DRM Rapid Screening Tool - Questionnaire.xlsx
@@ -90,7 +90,7 @@
     <t xml:space="preserve">Have any implementing decrees or regulations been approved since the adoption of the DRM legal framework? (e.g., rules on the structure or functions of the DRM agency or implementing regulations of the DRM law)</t>
   </si>
   <si>
-    <t xml:space="preserve">In the last 4 years, have DRM policy instruments reflecting progress towards the objective laid out in the DRM legal framework been officially approved/updated? (e.g., DRM strategies or policies) </t>
+    <t xml:space="preserve">In the last 5 years, have DRM policy instruments reflecting progress towards the objective laid out in the DRM legal framework been officially approved/updated? (e.g., DRM strategies or policies) </t>
   </si>
   <si>
     <t xml:space="preserve">Did the institution responsible for coordinating or leading DRM activities receive dedicated and significant funding for these functions in the last fiscal year? </t>
@@ -135,7 +135,7 @@
     <t xml:space="preserve">Do guidelines or procedures for managing housing/settlements located in high-risk areas exist?</t>
   </si>
   <si>
-    <t xml:space="preserve">In the past 4 years, has risk information (e.g., hazard maps, risk assessments) consistently informed the elaboration of territorial, spatial, land use or urban planning instruments? (e.g., more than 50% of urban plans approved include risk considerations)</t>
+    <t xml:space="preserve">In the past 5 years, has risk information (e.g., hazard maps, risk assessments) consistently informed the elaboration of territorial, spatial, land use or urban planning instruments? (e.g., more than 50% of urban plans approved include risk considerations)</t>
   </si>
   <si>
     <t xml:space="preserve">3.2. Public investment at the central level</t>
@@ -168,7 +168,7 @@
     <t xml:space="preserve">Is there at least one legally binding building code or standard that requires earthquake-resistant or other hazard-resistant (e.g., wind, flood) design for buildings?</t>
   </si>
   <si>
-    <t xml:space="preserve">In the past 4 years, has any public project or program been allocated funding for retrofitting activities that follow vulnerability assessments and resilient design standards?</t>
+    <t xml:space="preserve">In the past 5 years, has any public project or program been allocated funding for retrofitting activities that follow vulnerability assessments and resilient design standards?</t>
   </si>
   <si>
     <t xml:space="preserve">Is there a legal framework for water supply and sanitation in urban areas that take flood risk into account?</t>
@@ -177,7 +177,7 @@
     <t xml:space="preserve">Is there a water governance framework that includes a coordination mechanism gathering the main actors in charge of Integrated Water Resources Management (e.g., water, agriculture, urban planning, energy)?</t>
   </si>
   <si>
-    <t xml:space="preserve">Have any watershed basins undergone improvements in water management in the last four years?</t>
+    <t xml:space="preserve">Have any watershed basins undergone improvements in water management in the last 5 years?</t>
   </si>
   <si>
     <t xml:space="preserve">4. Preparedness</t>
@@ -192,7 +192,7 @@
     <t xml:space="preserve">Over the most recent major disaster, was the population promptly alerted (e.g., via SMS or other tailored communication channels)? </t>
   </si>
   <si>
-    <t xml:space="preserve">In the past 4 years, has there been a consistent budget allocation for the expansion, maintenance, and operation of the geophysical and/or hydrometeorological network?</t>
+    <t xml:space="preserve">In the past 5 years, has there been a consistent budget allocation for the expansion, maintenance, and operation of the geophysical and/or hydrometeorological network?</t>
   </si>
   <si>
     <t xml:space="preserve">4.2. Emergency Preparedness and Response (EP&amp;R)</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">Are there regulations that define standards for catastrophe insurance coverage of public or private assets?</t>
   </si>
   <si>
-    <t xml:space="preserve">In the past 4 years, has the $ amount of financing that can be mobilized through sovereign risk financing instruments increased?</t>
+    <t xml:space="preserve">In the past 5 years, has the $ amount of financing that can be mobilized through sovereign risk financing instruments increased?</t>
   </si>
   <si>
     <t xml:space="preserve">6. Resilient Reconstruction</t>

</xml_diff>

<commit_message>
feat: add diagnostic assessment documents and implement LLM knowledge base for public investment scoring
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Questionnaire.xlsx
+++ b/data/DRM Rapid Screening Tool - Questionnaire.xlsx
@@ -102,7 +102,7 @@
     <t xml:space="preserve">Does the National Development Strategy (or equivalent national planning instrument) contain objectives, targets or indicators related to DRM / DRR?</t>
   </si>
   <si>
-    <t xml:space="preserve">Have at least 4 essential government entities* included explicit DRM/ DRR targets and indicators in their most recent strategic planning documents? (e.g., Ministry of Health Strategic Plan, National Education Strategy/Policy, National Water and Sanitation Master Plan, Transport Infrastructure Development Plan)</t>
+    <t xml:space="preserve">Have at least 4 essential government entities* included explicit DRM/ DRR targets and indicators in their most recent strategic planning documents? (e.g., Ministry of Health Strategic Plan, National Education Strategy/Policy, Tourism Policy, National Water and Sanitation Master Plan, Transport Infrastructure Development Plan)</t>
   </si>
   <si>
     <t xml:space="preserve">2. Risk Identification</t>
@@ -141,10 +141,11 @@
     <t xml:space="preserve">3.2. Public investment at the central level</t>
   </si>
   <si>
-    <t xml:space="preserve">Do laws and regulations mandate disaster and climate risk screening as part of the appraisal of new public investment projects?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Do official guidelines exist defining disaster and climate risk screening methodologies for new public investment projects? </t>
+    <t xml:space="preserve">Do laws and regulations mandate disaster and climate risk screening as part of the appraisal of new public investment projects, including new Public-Private Partnerships?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the government provide incentives for private-sector actors (including tourism, retail, and property businesses) to invest in disaster-resilient infrastructure or business continuity planning?
+Examples of such incentives may include the promotion of business continuity planning, resilience standards linked to financing mechanisms, tax incentives, subsidies, or other forms of financial support.</t>
   </si>
   <si>
     <t xml:space="preserve">Are approved projects that have been identified as high-risk (or equivalent) through the disaster and climate screening process required to include risk mitigation measures?</t>
@@ -271,7 +272,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,6 +374,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -474,7 +481,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -613,6 +620,10 @@
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -898,7 +909,7 @@
   <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="2.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="89.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="3" width="31.44"/>
@@ -1560,7 +1571,7 @@
     <row r="30" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="24"/>
       <c r="C30" s="24"/>
-      <c r="D30" s="24" t="s">
+      <c r="D30" s="35" t="s">
         <v>40</v>
       </c>
       <c r="E30" s="29"/>
@@ -1606,7 +1617,7 @@
         <f aca="false">_xlfn.TEXTJOIN(";",FALSE(),J31,E31,H31)</f>
         <v>Q17;;1</v>
       </c>
-      <c r="L31" s="35"/>
+      <c r="L31" s="36"/>
     </row>
     <row r="32" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B32" s="24"/>
@@ -1638,7 +1649,7 @@
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B33" s="24"/>
       <c r="C33" s="24"/>
-      <c r="D33" s="36" t="s">
+      <c r="D33" s="37" t="s">
         <v>44</v>
       </c>
       <c r="E33" s="26"/>
@@ -1663,7 +1674,7 @@
     <row r="34" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="24"/>
       <c r="C34" s="24"/>
-      <c r="D34" s="37" t="s">
+      <c r="D34" s="38" t="s">
         <v>45</v>
       </c>
       <c r="E34" s="29"/>
@@ -1688,7 +1699,7 @@
     <row r="35" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B35" s="24"/>
       <c r="C35" s="24"/>
-      <c r="D35" s="36" t="s">
+      <c r="D35" s="37" t="s">
         <v>46</v>
       </c>
       <c r="E35" s="26"/>
@@ -1836,13 +1847,13 @@
       </c>
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B41" s="38" t="s">
+      <c r="B41" s="39" t="s">
         <v>52</v>
       </c>
       <c r="C41" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="D41" s="39" t="s">
+      <c r="D41" s="40" t="s">
         <v>54</v>
       </c>
       <c r="E41" s="26"/>
@@ -1865,9 +1876,9 @@
       </c>
     </row>
     <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B42" s="38"/>
+      <c r="B42" s="39"/>
       <c r="C42" s="24"/>
-      <c r="D42" s="40" t="s">
+      <c r="D42" s="41" t="s">
         <v>55</v>
       </c>
       <c r="E42" s="29"/>
@@ -1890,9 +1901,9 @@
       </c>
     </row>
     <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B43" s="38"/>
+      <c r="B43" s="39"/>
       <c r="C43" s="24"/>
-      <c r="D43" s="39" t="s">
+      <c r="D43" s="40" t="s">
         <v>56</v>
       </c>
       <c r="E43" s="26"/>
@@ -1915,11 +1926,11 @@
       </c>
     </row>
     <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B44" s="38"/>
+      <c r="B44" s="39"/>
       <c r="C44" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D44" s="40" t="s">
+      <c r="D44" s="41" t="s">
         <v>58</v>
       </c>
       <c r="E44" s="29"/>
@@ -1942,9 +1953,9 @@
       </c>
     </row>
     <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B45" s="38"/>
+      <c r="B45" s="39"/>
       <c r="C45" s="24"/>
-      <c r="D45" s="39" t="s">
+      <c r="D45" s="40" t="s">
         <v>59</v>
       </c>
       <c r="E45" s="26"/>
@@ -1967,9 +1978,9 @@
       </c>
     </row>
     <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B46" s="38"/>
+      <c r="B46" s="39"/>
       <c r="C46" s="24"/>
-      <c r="D46" s="40" t="s">
+      <c r="D46" s="41" t="s">
         <v>60</v>
       </c>
       <c r="E46" s="29"/>
@@ -1992,9 +2003,9 @@
       </c>
     </row>
     <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="38"/>
+      <c r="B47" s="39"/>
       <c r="C47" s="24"/>
-      <c r="D47" s="39" t="s">
+      <c r="D47" s="40" t="s">
         <v>61</v>
       </c>
       <c r="E47" s="26"/>
@@ -2017,11 +2028,11 @@
       </c>
     </row>
     <row r="48" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="38"/>
+      <c r="B48" s="39"/>
       <c r="C48" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="D48" s="40" t="s">
+      <c r="D48" s="41" t="s">
         <v>63</v>
       </c>
       <c r="E48" s="29"/>
@@ -2044,9 +2055,9 @@
       </c>
     </row>
     <row r="49" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B49" s="38"/>
+      <c r="B49" s="39"/>
       <c r="C49" s="24"/>
-      <c r="D49" s="39" t="s">
+      <c r="D49" s="40" t="s">
         <v>64</v>
       </c>
       <c r="E49" s="26"/>
@@ -2069,9 +2080,9 @@
       </c>
     </row>
     <row r="50" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B50" s="38"/>
+      <c r="B50" s="39"/>
       <c r="C50" s="24"/>
-      <c r="D50" s="40" t="s">
+      <c r="D50" s="41" t="s">
         <v>65</v>
       </c>
       <c r="E50" s="29"/>
@@ -2094,13 +2105,13 @@
       </c>
     </row>
     <row r="51" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B51" s="38" t="s">
+      <c r="B51" s="39" t="s">
         <v>66</v>
       </c>
       <c r="C51" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="D51" s="39" t="s">
+      <c r="D51" s="40" t="s">
         <v>68</v>
       </c>
       <c r="E51" s="26"/>
@@ -2123,9 +2134,9 @@
       </c>
     </row>
     <row r="52" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="38"/>
+      <c r="B52" s="39"/>
       <c r="C52" s="24"/>
-      <c r="D52" s="40" t="s">
+      <c r="D52" s="41" t="s">
         <v>69</v>
       </c>
       <c r="E52" s="29"/>
@@ -2148,9 +2159,9 @@
       </c>
     </row>
     <row r="53" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B53" s="38"/>
+      <c r="B53" s="39"/>
       <c r="C53" s="24"/>
-      <c r="D53" s="39" t="s">
+      <c r="D53" s="40" t="s">
         <v>70</v>
       </c>
       <c r="E53" s="26"/>
@@ -2173,9 +2184,9 @@
       </c>
     </row>
     <row r="54" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B54" s="38"/>
+      <c r="B54" s="39"/>
       <c r="C54" s="24"/>
-      <c r="D54" s="40" t="s">
+      <c r="D54" s="41" t="s">
         <v>71</v>
       </c>
       <c r="E54" s="29"/>
@@ -2198,11 +2209,11 @@
       </c>
     </row>
     <row r="55" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B55" s="38"/>
+      <c r="B55" s="39"/>
       <c r="C55" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="D55" s="39" t="s">
+      <c r="D55" s="40" t="s">
         <v>73</v>
       </c>
       <c r="E55" s="26"/>
@@ -2225,9 +2236,9 @@
       </c>
     </row>
     <row r="56" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B56" s="38"/>
+      <c r="B56" s="39"/>
       <c r="C56" s="24"/>
-      <c r="D56" s="40" t="s">
+      <c r="D56" s="41" t="s">
         <v>74</v>
       </c>
       <c r="E56" s="29"/>
@@ -2250,9 +2261,9 @@
       </c>
     </row>
     <row r="57" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B57" s="38"/>
+      <c r="B57" s="39"/>
       <c r="C57" s="24"/>
-      <c r="D57" s="39" t="s">
+      <c r="D57" s="40" t="s">
         <v>75</v>
       </c>
       <c r="E57" s="26"/>
@@ -2275,13 +2286,13 @@
       </c>
     </row>
     <row r="58" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B58" s="38" t="s">
+      <c r="B58" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="C58" s="38" t="s">
+      <c r="C58" s="39" t="s">
         <v>76</v>
       </c>
-      <c r="D58" s="40" t="s">
+      <c r="D58" s="41" t="s">
         <v>77</v>
       </c>
       <c r="E58" s="29"/>
@@ -2304,9 +2315,9 @@
       </c>
     </row>
     <row r="59" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B59" s="38"/>
-      <c r="C59" s="38"/>
-      <c r="D59" s="39" t="s">
+      <c r="B59" s="39"/>
+      <c r="C59" s="39"/>
+      <c r="D59" s="40" t="s">
         <v>78</v>
       </c>
       <c r="E59" s="26"/>
@@ -2329,9 +2340,9 @@
       </c>
     </row>
     <row r="60" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B60" s="38"/>
-      <c r="C60" s="38"/>
-      <c r="D60" s="40" t="s">
+      <c r="B60" s="39"/>
+      <c r="C60" s="39"/>
+      <c r="D60" s="41" t="s">
         <v>79</v>
       </c>
       <c r="E60" s="29"/>

</xml_diff>

<commit_message>
feat: modularize dashboard layout and incorporate project documentation and LLM narrative data.
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Questionnaire.xlsx
+++ b/data/DRM Rapid Screening Tool - Questionnaire.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="80">
   <si>
-    <t xml:space="preserve">Evaluating Disaster Risk Management Policy Frameworks: A Rapid Screening Tool</t>
+    <t xml:space="preserve">Evaluating Disaster Risk Management Policy Frameworks: A DRM Policy Diagnostic Tool</t>
   </si>
   <si>
     <t xml:space="preserve">Instructions</t>
@@ -272,7 +272,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -374,12 +374,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -622,7 +616,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2502,8 +2496,7 @@
     <row r="196" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="197" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B2:H2"/>
+  <mergeCells count="18">
     <mergeCell ref="B15:B20"/>
     <mergeCell ref="C15:C18"/>
     <mergeCell ref="C19:C20"/>

</xml_diff>

<commit_message>
Update DRM Rapid Screening Tool - Questionnaire.xlsx
</commit_message>
<xml_diff>
--- a/data/DRM Rapid Screening Tool - Questionnaire.xlsx
+++ b/data/DRM Rapid Screening Tool - Questionnaire.xlsx
@@ -141,10 +141,10 @@
     <t xml:space="preserve">3.2. Public investment at the central level</t>
   </si>
   <si>
-    <t xml:space="preserve">Do laws and regulations mandate disaster and climate risk screening as part of the appraisal of new public investment projects, including new Public-Private Partnerships?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Does the government provide incentives for private-sector actors (including tourism, retail, and property businesses) to invest in disaster-resilient infrastructure or business continuity planning?
+    <t xml:space="preserve">Do laws and regulations mandate disaster and climate risk screening as part of the appraisal of public investment projects, including Public-Private Partnerships?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the government provide incentives for private-sector actors (including tourism, retail, and property businesses) to invest in disaster-resilient infrastructure and/or business continuity planning?
 Examples of such incentives may include the promotion of business continuity planning, resilience standards linked to financing mechanisms, tax incentives, subsidies, or other forms of financial support.</t>
   </si>
   <si>

</xml_diff>